<commit_message>
:fried_egg: taxo correc° before datasets split => clean taxo names on 16S D1 LBM
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Dataset_1/ps_16S_cl_Dataset_1_tax_table.xlsx
+++ b/data/derived_data/2_RarefyData/Dataset_1/ps_16S_cl_Dataset_1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="414">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -816,6 +816,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cluster_337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tatumella</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_338</t>
@@ -3575,7 +3578,7 @@
         <v>24</v>
       </c>
       <c r="G77" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H77" t="s">
         <v>85</v>
@@ -4849,7 +4852,7 @@
         <v>29</v>
       </c>
       <c r="G126" t="s">
-        <v>15</v>
+        <v>268</v>
       </c>
       <c r="H126" t="s">
         <v>15</v>
@@ -4857,7 +4860,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -4875,15 +4878,15 @@
         <v>231</v>
       </c>
       <c r="G127" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H127" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -4901,7 +4904,7 @@
         <v>29</v>
       </c>
       <c r="G128" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H128" t="s">
         <v>15</v>
@@ -4909,7 +4912,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -4935,7 +4938,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -4953,7 +4956,7 @@
         <v>120</v>
       </c>
       <c r="G130" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H130" t="s">
         <v>15</v>
@@ -4961,7 +4964,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -4987,7 +4990,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -5005,7 +5008,7 @@
         <v>120</v>
       </c>
       <c r="G132" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H132" t="s">
         <v>15</v>
@@ -5013,7 +5016,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -5039,7 +5042,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -5054,10 +5057,10 @@
         <v>94</v>
       </c>
       <c r="F134" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G134" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H134" t="s">
         <v>15</v>
@@ -5065,7 +5068,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
@@ -5091,7 +5094,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -5117,7 +5120,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B137" t="s">
         <v>9</v>
@@ -5143,7 +5146,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -5164,12 +5167,12 @@
         <v>25</v>
       </c>
       <c r="H138" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -5184,18 +5187,18 @@
         <v>28</v>
       </c>
       <c r="F139" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G139" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H139" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -5221,7 +5224,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -5247,7 +5250,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -5273,7 +5276,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -5299,7 +5302,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -5325,7 +5328,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -5351,7 +5354,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -5366,18 +5369,18 @@
         <v>28</v>
       </c>
       <c r="F146" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G146" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H146" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -5395,7 +5398,7 @@
         <v>216</v>
       </c>
       <c r="G147" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H147" t="s">
         <v>15</v>
@@ -5403,7 +5406,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -5429,7 +5432,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -5455,7 +5458,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -5481,7 +5484,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -5507,7 +5510,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -5533,7 +5536,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -5559,7 +5562,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -5585,7 +5588,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -5611,7 +5614,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -5637,7 +5640,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -5658,12 +5661,12 @@
         <v>15</v>
       </c>
       <c r="H157" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -5689,7 +5692,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -5715,7 +5718,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -5727,13 +5730,13 @@
         <v>48</v>
       </c>
       <c r="E160" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F160" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G160" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H160" t="s">
         <v>15</v>
@@ -5741,7 +5744,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -5767,7 +5770,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -5793,7 +5796,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -5819,7 +5822,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -5837,7 +5840,7 @@
         <v>29</v>
       </c>
       <c r="G164" t="s">
-        <v>15</v>
+        <v>268</v>
       </c>
       <c r="H164" t="s">
         <v>15</v>
@@ -5845,7 +5848,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -5866,12 +5869,12 @@
         <v>25</v>
       </c>
       <c r="H165" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -5897,7 +5900,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
@@ -5923,7 +5926,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -5944,12 +5947,12 @@
         <v>25</v>
       </c>
       <c r="H168" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -5975,7 +5978,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -5987,13 +5990,13 @@
         <v>48</v>
       </c>
       <c r="E170" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F170" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G170" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="H170" t="s">
         <v>15</v>
@@ -6001,7 +6004,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -6027,7 +6030,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -6048,12 +6051,12 @@
         <v>233</v>
       </c>
       <c r="H172" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -6071,7 +6074,7 @@
         <v>135</v>
       </c>
       <c r="G173" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="H173" t="s">
         <v>15</v>
@@ -6079,7 +6082,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -6105,7 +6108,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B175" t="s">
         <v>15</v>
@@ -6131,7 +6134,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -6152,12 +6155,12 @@
         <v>15</v>
       </c>
       <c r="H176" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -6183,7 +6186,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -6209,7 +6212,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -6235,7 +6238,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -6261,7 +6264,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -6287,7 +6290,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -6313,7 +6316,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -6339,7 +6342,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -6365,7 +6368,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -6391,7 +6394,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -6417,7 +6420,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -6443,7 +6446,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -6469,7 +6472,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -6478,16 +6481,16 @@
         <v>47</v>
       </c>
       <c r="D189" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E189" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F189" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G189" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H189" t="s">
         <v>15</v>
@@ -6495,7 +6498,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -6513,7 +6516,7 @@
         <v>120</v>
       </c>
       <c r="G190" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H190" t="s">
         <v>15</v>
@@ -6521,7 +6524,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -6547,7 +6550,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
@@ -6573,7 +6576,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -6599,7 +6602,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -6625,7 +6628,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -6651,7 +6654,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -6666,18 +6669,18 @@
         <v>222</v>
       </c>
       <c r="F196" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G196" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H196" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -6703,7 +6706,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -6729,7 +6732,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -6755,7 +6758,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -6781,7 +6784,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -6799,7 +6802,7 @@
         <v>172</v>
       </c>
       <c r="G201" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="H201" t="s">
         <v>15</v>
@@ -6807,7 +6810,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -6833,7 +6836,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -6859,7 +6862,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -6880,12 +6883,12 @@
         <v>70</v>
       </c>
       <c r="H204" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -6911,7 +6914,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -6937,7 +6940,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -6963,7 +6966,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -6984,30 +6987,30 @@
         <v>15</v>
       </c>
       <c r="H208" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
       </c>
       <c r="C209" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D209" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E209" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F209" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G209" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H209" t="s">
         <v>15</v>
@@ -7015,7 +7018,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -7041,7 +7044,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -7067,7 +7070,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -7093,7 +7096,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -7119,7 +7122,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -7145,7 +7148,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -7171,7 +7174,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -7197,7 +7200,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -7223,7 +7226,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -7238,10 +7241,10 @@
         <v>33</v>
       </c>
       <c r="F218" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G218" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H218" t="s">
         <v>15</v>
@@ -7249,7 +7252,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -7275,7 +7278,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -7301,7 +7304,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -7327,7 +7330,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
@@ -7353,7 +7356,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -7379,7 +7382,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -7405,7 +7408,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -7431,7 +7434,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -7449,7 +7452,7 @@
         <v>24</v>
       </c>
       <c r="G226" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H226" t="s">
         <v>85</v>
@@ -7457,7 +7460,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -7475,7 +7478,7 @@
         <v>120</v>
       </c>
       <c r="G227" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H227" t="s">
         <v>15</v>
@@ -7483,7 +7486,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -7509,7 +7512,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -7535,7 +7538,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -7561,7 +7564,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -7587,7 +7590,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
:cow2::cow2:taxo manuammy specified before datasets split + suppr. alluvial plot part + special folder for old plots
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Dataset_1/ps_16S_cl_Dataset_1_tax_table.xlsx
+++ b/data/derived_data/2_RarefyData/Dataset_1/ps_16S_cl_Dataset_1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="415">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -1068,6 +1068,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cluster_6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gluconobacter cerinus</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_600</t>
@@ -3133,7 +3136,7 @@
         <v>28</v>
       </c>
       <c r="F60" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="G60" t="s">
         <v>15</v>
@@ -6467,12 +6470,12 @@
         <v>57</v>
       </c>
       <c r="H188" t="s">
-        <v>15</v>
+        <v>352</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -6481,16 +6484,16 @@
         <v>47</v>
       </c>
       <c r="D189" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E189" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F189" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G189" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H189" t="s">
         <v>15</v>
@@ -6498,7 +6501,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -6516,7 +6519,7 @@
         <v>120</v>
       </c>
       <c r="G190" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="H190" t="s">
         <v>15</v>
@@ -6524,7 +6527,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -6550,7 +6553,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
@@ -6576,7 +6579,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -6602,7 +6605,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -6628,7 +6631,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -6654,7 +6657,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -6669,18 +6672,18 @@
         <v>222</v>
       </c>
       <c r="F196" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G196" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H196" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -6706,7 +6709,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -6732,7 +6735,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -6758,7 +6761,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -6784,7 +6787,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -6802,7 +6805,7 @@
         <v>172</v>
       </c>
       <c r="G201" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H201" t="s">
         <v>15</v>
@@ -6810,7 +6813,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -6836,7 +6839,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -6862,7 +6865,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -6883,12 +6886,12 @@
         <v>70</v>
       </c>
       <c r="H204" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -6914,7 +6917,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -6940,7 +6943,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -6966,7 +6969,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -6987,30 +6990,30 @@
         <v>15</v>
       </c>
       <c r="H208" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
       </c>
       <c r="C209" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D209" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E209" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F209" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G209" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="H209" t="s">
         <v>15</v>
@@ -7018,7 +7021,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -7044,7 +7047,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -7070,7 +7073,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -7096,7 +7099,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -7122,7 +7125,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -7148,7 +7151,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -7174,7 +7177,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -7200,7 +7203,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -7226,7 +7229,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -7241,10 +7244,10 @@
         <v>33</v>
       </c>
       <c r="F218" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G218" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H218" t="s">
         <v>15</v>
@@ -7252,7 +7255,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -7278,7 +7281,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -7304,7 +7307,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -7330,7 +7333,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
@@ -7356,7 +7359,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -7382,7 +7385,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -7408,7 +7411,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -7434,7 +7437,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -7460,7 +7463,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -7486,7 +7489,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -7512,7 +7515,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -7538,7 +7541,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -7564,7 +7567,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -7590,7 +7593,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>

</xml_diff>